<commit_message>
Added steps to construct Hilbert envelopes, do PLS on those, fit OLS stat models (SM) to Hilbert STDs, plot SM fits on inflated brain
</commit_message>
<xml_diff>
--- a/description/processing.xlsx
+++ b/description/processing.xlsx
@@ -5,11 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Subjects" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="PLS" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="SM fits 1" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="SM fits 2" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="335">
   <si>
     <t xml:space="preserve">Subject ID</t>
   </si>
@@ -89,7 +91,7 @@
     <t xml:space="preserve">52C4TG</t>
   </si>
   <si>
-    <t xml:space="preserve">no bem</t>
+    <t xml:space="preserve">Not included into analysis done before Feb 6</t>
   </si>
   <si>
     <t xml:space="preserve">54RWW6</t>
@@ -1641,6 +1643,500 @@
       </rPr>
       <t xml:space="preserve">  0.44</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Stat model fitting results for 100 subjects, Hilbert envelope STD averaged over 1 – 2 s interval rel to image start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santa-Clara scores used as religiosity measure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For each fitted parameter, the following stats over ROIs are listed in brackets: (Mean, STD, Mean/STD, N signif ROIs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">God (111)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thing (121)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human (131)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super (141)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 – 7 Hz</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Group</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: pos, variable, peaks to 2. (1.10 0.40 2.76 2)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: pos, variable, peaks to 2.5. (1.15 0.50 2.32 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFC9211E"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Inter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: neg, variable, peaks to -2. (-1.23 0.42 -2.94 3)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Group</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: pos, smooth, peaks to 1.5 (0.90 0.26  3.47 0)
+SC: pos, smooth, rare peaks to 2.5 (1.39 0.32 4.39 3)
+Inter: neg, smooth, peaks to -2 (-1.24 0.23 -5.33 2)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Group</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: pos, smooth, larger then Thing,
+ peaks to 1.5
+ (1.26 0.27  4.64 1)
+SC: pos, variable, rare peaks to 2 (1.06 0.42 2.56 0)
+Inter: neg, smooth, peaks to -2 (-1.38 0.31 -4.46 3)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Group</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: pos, </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">highly variable, gaps</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, peaks to 2 (0.99 0.51 1.95 3)
+SC: pos, highly variable, smaller than others,
+peaks to 1.5 (0.49 0.45  1.08 0)
+Inter: neg, highly variable, smaller than others,
+peaks to -1.5 (-0.93 0.43 -2.13 0)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">8 – 13 Hz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, variable, peaks to 1.5
+SC: pos, variable, peaks to 1.5
+Inter: neg, variable, peaks to -1.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, smooth, lower level,
+Peaks to 1.5
+SC: pos, smooth, one peak to 2.5
+Inter: neg, smooth, peaks to -1.5,
+Single to -2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, LH smooth, RH variable,
+larger then Thing, peaks to 2.
+SC: pos, variable, low in RH, rare peaks
+to 1.5
+Inter: neg, LH smooth, RH variable,
+Peaks to -1.5</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Group: mostly pos, highly variable, </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">gaps</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, peaks to 2
+SC: sign alternating, highly variable, smaller
+than others, peaks to +1.5, -0.5.
+Inter: mostly neg, highly variable, 
+peaks to 1, -1.5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">14 – 21 Hz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, mod variable, peaks to
+1.5
+SC: pos, variable, peaks to 2
+Inter: neg, variable, peaks to -2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, mod variable, lower lev,
+Peaks to 1.5
+SC: pos, smooth, one peak to 2
+Inter: neg, smooth, peaks to -1.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, variable, larger then Thing,
+peaks to 2.5.
+SC: alternating, variable, more pos in RH,
+rare peaks to 1.5, -1
+Inter: neg, variable, peaks to -2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: mostly pos (more so in RH), highly
+variable, gaps in LH, peaks to 2
+SC: mostly pos esp in RH, highly variable,
+peaks to +2.
+Inter: neg, highly variable in LH, peaks -2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 – 28 Hz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, mod variable, peaks to
+1.5
+SC: pos, highly variable, small, peaks
+to 2
+Inter: neg, mod variable, peaks to -2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, mod variable, same lev
+as God, Peaks to 2.
+SC: pos, variable, peaks to 1.5
+Inter: neg, smooth, peaks to -1.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, mod variable, larger then Thing,
+peaks to 2.
+SC: pos, highly variable, peaks to 2.
+Inter: neg, smooth, peaks to -2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, highly variable, peaks to 2, many
+stat signif points
+SC: mostly pos highly variable, peaks to +2.
+Inter: neg, variable, peaks -2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 – 50 Hz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, mod variable, peaks to 1.5
+SC: mostly pos, highly variable, small,
+peaks to 1.5
+Inter: neg, mod variable, peaks to -2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, variable, same lev
+as God, Peaks to 2.
+SC: pos, highly variable, peaks to 1.5
+Inter: neg, variable, peaks to -1.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, smooth, larger then Thing,
+peaks to 2, many stat sign points.
+SC: pos, highly variable, peaks to 2.
+Inter: neg, smooth, peaks to -2, many stat 
+signif points.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group: pos, mod variable, peaks to 2.5, many
+stat signif points in RH
+SC: mostly pos highly variable, small, peaks
+around 1
+Inter: neg, mod variable, peaks -2.5, many stat
+signif points in RH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fits for a single image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pooled over frq bands quantiles for 2-sided alpha = 0.01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lower</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cbar lims</t>
+  </si>
+  <si>
+    <t xml:space="preserve">group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.4, 2.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.8, 2.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">group*rel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.5, 0.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lower threshold hits for group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upper threshold hits for group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ijob</t>
+  </si>
+  <si>
+    <t xml:space="preserve">band</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image(s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plotted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[4.0,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[8.0,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[14.0,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[21.0,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28.0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[30.0,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lower threshold hits for religion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upper threshold hits for religion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lower threshold hits for group*rel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upper threshold hits for group*rel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTE: in all cases just a single view is enough</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTE: in all cases just a single view is enough except for #7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fits for pairs of images</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.4, 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.9,1.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[4.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">141]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[111,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">131]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[121</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[121,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[131</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[8.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[14.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[30.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">121]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[131,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTE: 1 – 22 deep areas, small spots; 25,27,28  &gt;=2 areas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTE: 2,5,8,9,11 – two areas;</t>
   </si>
 </sst>
 </file>
@@ -1790,7 +2286,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1861,6 +2357,26 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1946,9 +2462,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>657000</xdr:colOff>
+      <xdr:colOff>655200</xdr:colOff>
       <xdr:row>80</xdr:row>
-      <xdr:rowOff>159840</xdr:rowOff>
+      <xdr:rowOff>158040</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1958,7 +2474,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10055520" y="10559160"/>
-          <a:ext cx="4857120" cy="3049920"/>
+          <a:ext cx="4854960" cy="3048120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2860,12 +3376,17 @@
       <c r="E12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
       <c r="L12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4504,12 +5025,17 @@
       <c r="E80" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F80" s="4" t="s">
+      <c r="F80" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="4"/>
+      <c r="H80" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I80" s="4"/>
+      <c r="J80" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G80" s="4"/>
-      <c r="H80" s="4"/>
-      <c r="I80" s="4"/>
       <c r="L80" s="4"/>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5417,7 +5943,7 @@
       </c>
       <c r="F115" s="2" t="n">
         <f aca="false">SUM(F2:F114)</f>
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G115" s="2" t="n">
         <f aca="false">SUM(G2:G114)</f>
@@ -5425,7 +5951,7 @@
       </c>
       <c r="H115" s="2" t="n">
         <f aca="false">SUM(H2:H114)</f>
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I115" s="2" t="n">
         <f aca="false">SUM(I2:I114)</f>
@@ -7727,4 +8253,2014 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="33.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="36.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="38.83"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="70.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="82.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>267</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="47.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>270</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>271</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="59.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>275</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>276</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>277</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="70.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>280</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>282</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>283</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M81"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18"/>
+      <c r="B3" s="19" t="s">
+        <v>286</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>287</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="B4" s="18" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="C4" s="18" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
+        <v>291</v>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19" t="s">
+        <v>293</v>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>-2.25</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="G8" s="2" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="C9" s="18"/>
+      <c r="D9" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="F9" s="18"/>
+      <c r="G9" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="H9" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="I9" s="18"/>
+      <c r="J9" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="K9" s="19" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>301</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>141</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="I10" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="J10" s="18" t="n">
+        <v>141</v>
+      </c>
+      <c r="K10" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>303</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>304</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>111</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="18"/>
+      <c r="G11" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="I11" s="21" t="s">
+        <v>306</v>
+      </c>
+      <c r="J11" s="21" t="n">
+        <v>131</v>
+      </c>
+      <c r="K11" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>121</v>
+      </c>
+      <c r="E12" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="18"/>
+      <c r="G12" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>307</v>
+      </c>
+      <c r="I12" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="J12" s="20" t="n">
+        <v>141</v>
+      </c>
+      <c r="K12" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>131</v>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="H13" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="I13" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="J13" s="18" t="n">
+        <v>131</v>
+      </c>
+      <c r="K13" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>141</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18" t="n">
+        <v>19</v>
+      </c>
+      <c r="H14" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="I14" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="J14" s="18" t="n">
+        <v>141</v>
+      </c>
+      <c r="K14" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>121</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="H18" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="I18" s="19"/>
+      <c r="J18" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="K18" s="19" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D19" s="18" t="n">
+        <v>111</v>
+      </c>
+      <c r="E19" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="18"/>
+      <c r="G19" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="20" t="s">
+        <v>301</v>
+      </c>
+      <c r="I19" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="J19" s="20" t="n">
+        <v>111</v>
+      </c>
+      <c r="K19" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <v>141</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="18"/>
+      <c r="G20" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="20" t="s">
+        <v>301</v>
+      </c>
+      <c r="I20" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="J20" s="20" t="n">
+        <v>121</v>
+      </c>
+      <c r="K20" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>305</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="D21" s="20" t="n">
+        <v>131</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="H21" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="I21" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="J21" s="18" t="n">
+        <v>121</v>
+      </c>
+      <c r="K21" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="D22" s="18" t="n">
+        <v>141</v>
+      </c>
+      <c r="E22" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="H22" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="I22" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="J22" s="18" t="n">
+        <v>111</v>
+      </c>
+      <c r="K22" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>111</v>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="H23" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="I23" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="J23" s="18" t="n">
+        <v>131</v>
+      </c>
+      <c r="K23" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="D24" s="18" t="n">
+        <v>111</v>
+      </c>
+      <c r="E24" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="H24" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="I24" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="J24" s="18" t="n">
+        <v>141</v>
+      </c>
+      <c r="K24" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="D25" s="18" t="n">
+        <v>121</v>
+      </c>
+      <c r="E25" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="18"/>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="D26" s="20" t="n">
+        <v>141</v>
+      </c>
+      <c r="E26" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="18"/>
+      <c r="J26" s="18"/>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="29" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="F29" s="19"/>
+      <c r="G29" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="H29" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="I29" s="19"/>
+      <c r="J29" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="K29" s="19" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="D30" s="18" t="n">
+        <v>111</v>
+      </c>
+      <c r="E30" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="H30" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="I30" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="J30" s="18" t="n">
+        <v>111</v>
+      </c>
+      <c r="K30" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="D31" s="18" t="n">
+        <v>141</v>
+      </c>
+      <c r="E31" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="18"/>
+      <c r="G31" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="H31" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="I31" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="J31" s="18" t="n">
+        <v>131</v>
+      </c>
+      <c r="K31" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="D32" s="18" t="n">
+        <v>131</v>
+      </c>
+      <c r="E32" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="18"/>
+      <c r="G32" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="H32" s="20" t="s">
+        <v>303</v>
+      </c>
+      <c r="I32" s="20" t="s">
+        <v>304</v>
+      </c>
+      <c r="J32" s="20" t="n">
+        <v>141</v>
+      </c>
+      <c r="K32" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="18" t="n">
+        <v>19</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="D33" s="18" t="n">
+        <v>141</v>
+      </c>
+      <c r="E33" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18" t="n">
+        <v>17</v>
+      </c>
+      <c r="H33" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="I33" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="J33" s="18" t="n">
+        <v>121</v>
+      </c>
+      <c r="K33" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="H34" s="18"/>
+      <c r="I34" s="18"/>
+      <c r="J34" s="18"/>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="6"/>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="22"/>
+      <c r="B40" s="19" t="s">
+        <v>286</v>
+      </c>
+      <c r="C40" s="19" t="s">
+        <v>287</v>
+      </c>
+      <c r="D40" s="19" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="B41" s="18" t="n">
+        <v>-1.35</v>
+      </c>
+      <c r="C41" s="18" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="D41" s="18" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="19" t="s">
+        <v>291</v>
+      </c>
+      <c r="B42" s="18" t="n">
+        <v>-2</v>
+      </c>
+      <c r="C42" s="18" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="D42" s="18"/>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="19" t="s">
+        <v>293</v>
+      </c>
+      <c r="B43" s="18" t="n">
+        <v>-1.81</v>
+      </c>
+      <c r="C43" s="18" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="D43" s="18" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="B45" s="2"/>
+      <c r="H45" s="2" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="B46" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="E46" s="18"/>
+      <c r="F46" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="H46" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="I46" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="J46" s="19"/>
+      <c r="K46" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="L46" s="18"/>
+      <c r="M46" s="19" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="C47" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="D47" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E47" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F47" s="18"/>
+      <c r="H47" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="J47" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="K47" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L47" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="M47" s="18"/>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B48" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="C48" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="D48" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="E48" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F48" s="18"/>
+      <c r="H48" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="I48" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="J48" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="K48" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="L48" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="M48" s="18"/>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="C49" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="D49" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="E49" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F49" s="18"/>
+      <c r="H49" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="I49" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="J49" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="K49" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L49" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="M49" s="18"/>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="B50" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="C50" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D50" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="E50" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F50" s="18"/>
+      <c r="H50" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="I50" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="J50" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="K50" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L50" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="M50" s="18"/>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="B51" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="C51" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="D51" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E51" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="F51" s="18"/>
+      <c r="H51" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="I51" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="J51" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="K51" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L51" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="M51" s="18"/>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B52" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="C52" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="D52" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="E52" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F52" s="18"/>
+      <c r="H52" s="18" t="n">
+        <v>26</v>
+      </c>
+      <c r="I52" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="J52" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="K52" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L52" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="M52" s="18"/>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="18" t="n">
+        <v>24</v>
+      </c>
+      <c r="B53" s="18" t="s">
+        <v>330</v>
+      </c>
+      <c r="C53" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="D53" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E53" s="18" t="s">
+        <v>331</v>
+      </c>
+      <c r="F53" s="18"/>
+      <c r="H53" s="18" t="n">
+        <v>27</v>
+      </c>
+      <c r="I53" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="J53" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="K53" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="L53" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="M53" s="18"/>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="18" t="n">
+        <v>29</v>
+      </c>
+      <c r="B54" s="18" t="s">
+        <v>330</v>
+      </c>
+      <c r="C54" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="D54" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="E54" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F54" s="18"/>
+      <c r="H54" s="18" t="n">
+        <v>28</v>
+      </c>
+      <c r="I54" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="J54" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="K54" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="L54" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="M54" s="18"/>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="B57" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="C57" s="19"/>
+      <c r="D57" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="E57" s="18"/>
+      <c r="H57" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="I57" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="J57" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="K57" s="18"/>
+      <c r="L57" s="18"/>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B58" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="C58" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="D58" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="E58" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="H58" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I58" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="J58" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="K58" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L58" s="18" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B59" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="C59" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="D59" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E59" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="H59" s="18" t="n">
+        <v>16</v>
+      </c>
+      <c r="I59" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="J59" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="K59" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="L59" s="18" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B60" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="C60" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="D60" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E60" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="H60" s="18" t="n">
+        <v>17</v>
+      </c>
+      <c r="I60" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="J60" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="K60" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="L60" s="18" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B61" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="C61" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="D61" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="E61" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="H61" s="18" t="n">
+        <v>19</v>
+      </c>
+      <c r="I61" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="J61" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="K61" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L61" s="18" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="B62" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C62" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D62" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E62" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="H62" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="I62" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="J62" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="K62" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="L62" s="18" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="B63" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="C63" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="D63" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="E63" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="H63" s="18" t="n">
+        <v>24</v>
+      </c>
+      <c r="I63" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="J63" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="K63" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L63" s="18" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="B64" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="C64" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="D64" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="E64" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="H64" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="I64" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="J64" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="K64" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L64" s="18" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="18" t="n">
+        <v>29</v>
+      </c>
+      <c r="B65" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="C65" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="D65" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="E65" s="18" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
+      <c r="D67" s="2"/>
+      <c r="E67" s="2"/>
+      <c r="F67" s="2"/>
+      <c r="H67" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="I67" s="2"/>
+      <c r="J67" s="2"/>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="B68" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="D68" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="E68" s="19"/>
+      <c r="F68" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="H68" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="I68" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="K68" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="L68" s="18"/>
+      <c r="M68" s="19" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B69" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="C69" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="D69" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="E69" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="F69" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H69" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I69" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="J69" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="K69" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L69" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="M69" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="B70" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="C70" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="D70" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="E70" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F70" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="I70" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="J70" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="K70" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="L70" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="M70" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B71" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="C71" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="D71" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="E71" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F71" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H71" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="I71" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="J71" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="K71" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="L71" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="M71" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="18" t="n">
+        <v>19</v>
+      </c>
+      <c r="B72" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="C72" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="D72" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="E72" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="F72" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="I72" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="J72" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="K72" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L72" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="M72" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="B73" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="C73" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="D73" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="E73" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F73" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="I73" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="J73" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="K73" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="L73" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="M73" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="18" t="n">
+        <v>22</v>
+      </c>
+      <c r="B74" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="C74" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="D74" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E74" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F74" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H74" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="I74" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="J74" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="K74" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="L74" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="M74" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="B75" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="C75" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="D75" s="20" t="s">
+        <v>323</v>
+      </c>
+      <c r="E75" s="20" t="s">
+        <v>324</v>
+      </c>
+      <c r="F75" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="I75" s="20" t="s">
+        <v>303</v>
+      </c>
+      <c r="J75" s="20" t="s">
+        <v>304</v>
+      </c>
+      <c r="K75" s="20" t="s">
+        <v>332</v>
+      </c>
+      <c r="L75" s="20" t="s">
+        <v>322</v>
+      </c>
+      <c r="M75" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="20" t="n">
+        <v>27</v>
+      </c>
+      <c r="B76" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="C76" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="D76" s="20" t="s">
+        <v>326</v>
+      </c>
+      <c r="E76" s="20" t="s">
+        <v>324</v>
+      </c>
+      <c r="F76" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="I76" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="J76" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="K76" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L76" s="18" t="s">
+        <v>331</v>
+      </c>
+      <c r="M76" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="B77" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="C77" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="D77" s="20" t="s">
+        <v>326</v>
+      </c>
+      <c r="E77" s="20" t="s">
+        <v>322</v>
+      </c>
+      <c r="F77" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="I77" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="J77" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="K77" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L77" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="M77" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="0" t="s">
+        <v>333</v>
+      </c>
+      <c r="H78" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="I78" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="J78" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="K78" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="L78" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="M78" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H79" s="18" t="n">
+        <v>24</v>
+      </c>
+      <c r="I79" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="J79" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="K79" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="L79" s="18" t="s">
+        <v>331</v>
+      </c>
+      <c r="M79" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H81" s="0" t="s">
+        <v>334</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>